<commit_message>
scope cookie to path
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/02a-cookies.xlsx
+++ b/translations/welsh-translations/xlsx/02a-cookies.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="124">
   <si>
     <t>Translator notes</t>
   </si>
@@ -305,6 +305,12 @@
   </si>
   <si>
     <t>Helps us understand how many people use the service by distinguishing individual users</t>
+  </si>
+  <si>
+    <t>cookies.analytics.gidPurpose</t>
+  </si>
+  <si>
+    <t>Helps us distinguish users during a browsing session</t>
   </si>
   <si>
     <t>cookies.analytics.gaContainerPurpose</t>
@@ -775,7 +781,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -1540,7 +1546,7 @@
         <v>105</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>106</v>
+        <v>14</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>14</v>
@@ -1548,19 +1554,19 @@
     </row>
     <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D42" s="1" t="s">
+      <c r="E42" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>14</v>
@@ -1568,19 +1574,19 @@
     </row>
     <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B43" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D43" s="1" t="s">
+      <c r="E43" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>112</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>14</v>
@@ -1588,19 +1594,19 @@
     </row>
     <row r="44" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D44" s="1" t="s">
+      <c r="E44" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>14</v>
@@ -1608,19 +1614,19 @@
     </row>
     <row r="45" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B45" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D45" s="1" t="s">
+      <c r="E45" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>14</v>
@@ -1628,26 +1634,46 @@
     </row>
     <row r="46" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B46" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D46" s="1" t="s">
+      <c r="E46" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="F46" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="B47" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:F46"/>
+  <autoFilter ref="A5:F47"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>

<commit_message>
MO-516: updqte welsh content
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/02a-cookies.xlsx
+++ b/translations/welsh-translations/xlsx/02a-cookies.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="130">
   <si>
     <t>Translator notes</t>
   </si>
@@ -103,22 +103,34 @@
     <t>Analytics cookies</t>
   </si>
   <si>
+    <t>Cwcis dadansoddi</t>
+  </si>
+  <si>
     <t>cookies.analyticsCookiesDescription1</t>
   </si>
   <si>
-    <t>We use Google Analytics to collect information about how you use this service.</t>
+    <t>With your permission, we use Google Analytics to collect information about how you use this service.</t>
+  </si>
+  <si>
+    <t>Gyda’ch caniatâd, rydym yn defnyddio Google Analytics i gasglu gwybodaeth am sut rydych chi'n defnyddio'r gwasanaeth yma.</t>
   </si>
   <si>
     <t>cookies.analyticsCookiesDescription2</t>
   </si>
   <si>
-    <t>We do this to help us understand how the service is being used and to make improvements.</t>
+    <t>This information helps us to improve our service.</t>
+  </si>
+  <si>
+    <t>Mae’r wybodaeth yma yn ein helpu i wella’n gwasanaeth.</t>
   </si>
   <si>
     <t>cookies.analyticsCookiesDescription3</t>
   </si>
   <si>
-    <t>Google Analytics stores information about:</t>
+    <t>Google Analytics cookies store information about:</t>
+  </si>
+  <si>
+    <t>Mae cwcis Google Analytics yn cadw gwybodaeth am:</t>
   </si>
   <si>
     <t>cookies.analyticsCookiesPoint1</t>
@@ -145,12 +157,18 @@
     <t>how you arrived at the service</t>
   </si>
   <si>
+    <t>sut y gwnaethoch chi gyrraedd y gwasanaeth</t>
+  </si>
+  <si>
     <t>cookies.analyticsCookiesPoint4</t>
   </si>
   <si>
     <t>what you click on while using the service</t>
   </si>
   <si>
+    <t>beth rydych chi’n clicio arno wrth ymweld â'r gwasanaeth</t>
+  </si>
+  <si>
     <t>cookies.analyticsCookiesPoint5</t>
   </si>
   <si>
@@ -160,12 +178,6 @@
     <t>y ddyfais a’r porwr rydych chi’n eu defnyddio</t>
   </si>
   <si>
-    <t>cookies.analyticsCookiesPermission</t>
-  </si>
-  <si>
-    <t>We only set Google Analytics cookies if you give us permission.</t>
-  </si>
-  <si>
     <t>cookies.table.essentialCookiesWeUse</t>
   </si>
   <si>
@@ -304,19 +316,19 @@
     <t>cookies.analytics.gaPurpose</t>
   </si>
   <si>
-    <t>Helps us understand how many people use the service by distinguishing individual users</t>
-  </si>
-  <si>
-    <t>cookies.analytics.gidPurpose</t>
-  </si>
-  <si>
-    <t>Helps us distinguish users during a browsing session</t>
+    <t>Counts individual visits to the service</t>
+  </si>
+  <si>
+    <t>Cyfri ymweliadau unigol â’r gwasanaeth</t>
   </si>
   <si>
     <t>cookies.analytics.gaContainerPurpose</t>
   </si>
   <si>
-    <t>Helps Google Analytics maintain information about your session</t>
+    <t>Tracks activity in a session</t>
+  </si>
+  <si>
+    <t>Olrhain gweithgarwch mewn sesiwn</t>
   </si>
   <si>
     <t>cookies.analytics.gaExpires</t>
@@ -325,10 +337,16 @@
     <t>2 years</t>
   </si>
   <si>
+    <t>2 flynedd</t>
+  </si>
+  <si>
     <t>cookies.settings.heading</t>
   </si>
   <si>
     <t>Change your cookie settings</t>
+  </si>
+  <si>
+    <t>Newid eich gosodiadau cwcis</t>
   </si>
   <si>
     <t>cookies.settings.legend</t>
@@ -781,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -966,15 +984,15 @@
         <v>29</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>10</v>
@@ -983,10 +1001,10 @@
         <v>11</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>14</v>
@@ -994,7 +1012,7 @@
     </row>
     <row r="14" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>10</v>
@@ -1003,10 +1021,10 @@
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>14</v>
@@ -1014,7 +1032,7 @@
     </row>
     <row r="15" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>10</v>
@@ -1023,10 +1041,10 @@
         <v>11</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>14</v>
@@ -1034,7 +1052,7 @@
     </row>
     <row r="16" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>10</v>
@@ -1043,10 +1061,10 @@
         <v>11</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>14</v>
@@ -1054,7 +1072,7 @@
     </row>
     <row r="17" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>10</v>
@@ -1063,10 +1081,10 @@
         <v>11</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>14</v>
@@ -1074,7 +1092,7 @@
     </row>
     <row r="18" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>10</v>
@@ -1083,10 +1101,10 @@
         <v>11</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>14</v>
@@ -1094,7 +1112,7 @@
     </row>
     <row r="19" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>10</v>
@@ -1103,10 +1121,10 @@
         <v>11</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>14</v>
@@ -1114,7 +1132,7 @@
     </row>
     <row r="20" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>10</v>
@@ -1123,10 +1141,10 @@
         <v>11</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>14</v>
@@ -1134,7 +1152,7 @@
     </row>
     <row r="21" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>10</v>
@@ -1143,10 +1161,10 @@
         <v>11</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>14</v>
@@ -1154,7 +1172,7 @@
     </row>
     <row r="22" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>10</v>
@@ -1163,10 +1181,10 @@
         <v>11</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>14</v>
@@ -1174,7 +1192,7 @@
     </row>
     <row r="23" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>10</v>
@@ -1183,10 +1201,10 @@
         <v>11</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>14</v>
@@ -1194,7 +1212,7 @@
     </row>
     <row r="24" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>10</v>
@@ -1203,10 +1221,10 @@
         <v>11</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>14</v>
@@ -1214,7 +1232,7 @@
     </row>
     <row r="25" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>10</v>
@@ -1223,10 +1241,10 @@
         <v>11</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>14</v>
@@ -1234,7 +1252,7 @@
     </row>
     <row r="26" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>10</v>
@@ -1243,10 +1261,10 @@
         <v>11</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>14</v>
@@ -1254,7 +1272,7 @@
     </row>
     <row r="27" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>10</v>
@@ -1263,10 +1281,10 @@
         <v>11</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>14</v>
@@ -1274,7 +1292,7 @@
     </row>
     <row r="28" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>10</v>
@@ -1283,10 +1301,10 @@
         <v>11</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>14</v>
@@ -1294,7 +1312,7 @@
     </row>
     <row r="29" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>10</v>
@@ -1303,10 +1321,10 @@
         <v>11</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>14</v>
@@ -1314,7 +1332,7 @@
     </row>
     <row r="30" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>10</v>
@@ -1323,10 +1341,10 @@
         <v>11</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>14</v>
@@ -1334,7 +1352,7 @@
     </row>
     <row r="31" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>10</v>
@@ -1343,10 +1361,10 @@
         <v>11</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>14</v>
@@ -1354,7 +1372,7 @@
     </row>
     <row r="32" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>10</v>
@@ -1363,10 +1381,10 @@
         <v>11</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>14</v>
@@ -1374,7 +1392,7 @@
     </row>
     <row r="33" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>10</v>
@@ -1383,10 +1401,10 @@
         <v>11</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>14</v>
@@ -1394,7 +1412,7 @@
     </row>
     <row r="34" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>10</v>
@@ -1403,10 +1421,10 @@
         <v>11</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>14</v>
@@ -1414,7 +1432,7 @@
     </row>
     <row r="35" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>10</v>
@@ -1423,10 +1441,10 @@
         <v>11</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>14</v>
@@ -1434,7 +1452,7 @@
     </row>
     <row r="36" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>10</v>
@@ -1443,10 +1461,10 @@
         <v>11</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>14</v>
@@ -1454,7 +1472,7 @@
     </row>
     <row r="37" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>10</v>
@@ -1463,10 +1481,10 @@
         <v>11</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>14</v>
+        <v>105</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>14</v>
@@ -1474,7 +1492,7 @@
     </row>
     <row r="38" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>10</v>
@@ -1483,10 +1501,10 @@
         <v>11</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>14</v>
+        <v>108</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>14</v>
@@ -1494,7 +1512,7 @@
     </row>
     <row r="39" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>10</v>
@@ -1503,10 +1521,10 @@
         <v>11</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>14</v>
@@ -1514,7 +1532,7 @@
     </row>
     <row r="40" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>10</v>
@@ -1523,10 +1541,10 @@
         <v>11</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>14</v>
+        <v>114</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>14</v>
@@ -1534,7 +1552,7 @@
     </row>
     <row r="41" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>10</v>
@@ -1543,10 +1561,10 @@
         <v>11</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>14</v>
+        <v>117</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>14</v>
@@ -1554,7 +1572,7 @@
     </row>
     <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>10</v>
@@ -1563,10 +1581,10 @@
         <v>11</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>14</v>
@@ -1574,7 +1592,7 @@
     </row>
     <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>10</v>
@@ -1583,10 +1601,10 @@
         <v>11</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>14</v>
@@ -1594,7 +1612,7 @@
     </row>
     <row r="44" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>10</v>
@@ -1603,10 +1621,10 @@
         <v>11</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>14</v>
@@ -1614,7 +1632,7 @@
     </row>
     <row r="45" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>10</v>
@@ -1623,63 +1641,23 @@
         <v>11</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="46" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="47" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:F47"/>
+  <autoFilter ref="A5:F45"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="D3:F3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: add missing translations
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/02a-cookies.xlsx
+++ b/translations/welsh-translations/xlsx/02a-cookies.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="133">
   <si>
     <t>Translator notes</t>
   </si>
@@ -232,6 +232,24 @@
     <t>Yn cynnal eich sesiwn ochr gweinydd wedi’i dilysu</t>
   </si>
   <si>
+    <t>cookies.ttl.day</t>
+  </si>
+  <si>
+    <t>1 day</t>
+  </si>
+  <si>
+    <t>1 diwrnod</t>
+  </si>
+  <si>
+    <t>cookies.ttl.days</t>
+  </si>
+  <si>
+    <t>{{count}} days</t>
+  </si>
+  <si>
+    <t>{{count}} diwrnod</t>
+  </si>
+  <si>
     <t>cookies.ttl.hour</t>
   </si>
   <si>
@@ -329,15 +347,6 @@
   </si>
   <si>
     <t>Olrhain gweithgarwch mewn sesiwn</t>
-  </si>
-  <si>
-    <t>cookies.analytics.gaExpires</t>
-  </si>
-  <si>
-    <t>2 years</t>
-  </si>
-  <si>
-    <t>2 flynedd</t>
   </si>
   <si>
     <t>cookies.settings.heading</t>
@@ -799,7 +808,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -1650,14 +1659,34 @@
         <v>14</v>
       </c>
     </row>
+    <row r="46" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:F45"/>
+  <autoFilter ref="A5:F46"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="D3:F3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>